<commit_message>
feat: Align EB contacts and Customers data sheets in Tables (1).xlsx with all registration form fields
</commit_message>
<xml_diff>
--- a/Tables (1).xlsx
+++ b/Tables (1).xlsx
@@ -38057,7 +38057,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:O36"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -38067,19 +38067,43 @@
         <v>Company name</v>
       </c>
       <c r="C1" t="str">
-        <v>Location</v>
+        <v>Circle</v>
       </c>
       <c r="D1" t="str">
+        <v>BA Name</v>
+      </c>
+      <c r="E1" t="str">
         <v>Contact name</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Designation</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Contact no</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>mail id</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Service Type</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Installation Address</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Bandwidth / Plan</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Circuit ID</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Billing Account No</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Date of Commission</v>
+      </c>
+      <c r="O1" t="str">
+        <v>WAN IP Address</v>
       </c>
     </row>
     <row r="2">
@@ -38092,16 +38116,16 @@
       <c r="C2" t="str">
         <v>Inavolu-Amaravathi</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>Ramu Nalluri</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>IT Manager</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>9618599503</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>it.manager@vitap.ac.in</v>
       </c>
     </row>
@@ -38115,16 +38139,16 @@
       <c r="C3" t="str">
         <v>Inavolu-Amaravathi</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>Nanda Kumar</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
         <v>Deputy Director</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
         <v>9840909833</v>
       </c>
-      <c r="G3" t="str">
+      <c r="H3" t="str">
         <v>deputydir.cts@vitap.ac.in</v>
       </c>
     </row>
@@ -38138,16 +38162,16 @@
       <c r="C4" t="str">
         <v>Inavolu-Amaravathi</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <v>Suresh</v>
       </c>
-      <c r="E4" t="str">
+      <c r="F4" t="str">
         <v>Purchase Manager</v>
       </c>
-      <c r="F4" t="str">
+      <c r="G4" t="str">
         <v>9533343625</v>
       </c>
-      <c r="G4" t="str">
+      <c r="H4" t="str">
         <v>purchase@vitap.ac.in</v>
       </c>
     </row>
@@ -38161,13 +38185,13 @@
       <c r="C5" t="str">
         <v>Inavolu-Amaravathi</v>
       </c>
-      <c r="D5" t="str">
+      <c r="E5" t="str">
         <v>Bhanu</v>
       </c>
-      <c r="E5" t="str">
+      <c r="F5" t="str">
         <v>Receptionist</v>
       </c>
-      <c r="F5" t="str">
+      <c r="G5" t="str">
         <v>0863-2370922</v>
       </c>
     </row>
@@ -38181,13 +38205,13 @@
       <c r="C6" t="str">
         <v>VIT Vellore</v>
       </c>
-      <c r="D6" t="str">
+      <c r="E6" t="str">
         <v>Yuvaraj</v>
       </c>
-      <c r="E6" t="str">
+      <c r="F6" t="str">
         <v>Director PA</v>
       </c>
-      <c r="F6" t="str">
+      <c r="G6" t="str">
         <v>9894660141</v>
       </c>
     </row>
@@ -38201,13 +38225,13 @@
       <c r="C7" t="str">
         <v>Inavolu-Amaravathi</v>
       </c>
-      <c r="D7" t="str">
+      <c r="E7" t="str">
         <v>Venkata krishna</v>
       </c>
-      <c r="E7" t="str">
+      <c r="F7" t="str">
         <v>Purchase sims</v>
       </c>
-      <c r="F7" t="str">
+      <c r="G7" t="str">
         <v>7780506556</v>
       </c>
     </row>
@@ -38221,13 +38245,13 @@
       <c r="C8" t="str">
         <v>Inavolu-Amaravathi</v>
       </c>
-      <c r="D8" t="str">
+      <c r="E8" t="str">
         <v>Suresh</v>
       </c>
-      <c r="E8" t="str">
+      <c r="F8" t="str">
         <v>Asst Manager</v>
       </c>
-      <c r="F8" t="str">
+      <c r="G8" t="str">
         <v>9444269837</v>
       </c>
     </row>
@@ -38241,16 +38265,16 @@
       <c r="C9" t="str">
         <v>Inavolu-Amaravathi</v>
       </c>
-      <c r="D9" t="str">
+      <c r="E9" t="str">
         <v>Poornima L</v>
       </c>
-      <c r="E9" t="str">
+      <c r="F9" t="str">
         <v>Manager  IT-Bills</v>
       </c>
-      <c r="F9" t="str">
+      <c r="G9" t="str">
         <v>9600160077</v>
       </c>
-      <c r="G9" t="str">
+      <c r="H9" t="str">
         <v>poornima.l@srmap.edu.in</v>
       </c>
     </row>
@@ -38264,16 +38288,16 @@
       <c r="C10" t="str">
         <v>Inavolu-Amaravathi</v>
       </c>
-      <c r="D10" t="str">
+      <c r="E10" t="str">
         <v>Suhasini</v>
       </c>
-      <c r="E10" t="str">
+      <c r="F10" t="str">
         <v>Asst Director</v>
       </c>
-      <c r="F10" t="str">
+      <c r="G10" t="str">
         <v>7397265412</v>
       </c>
-      <c r="G10" t="str">
+      <c r="H10" t="str">
         <v>suhasini.b@srmap.edu.in</v>
       </c>
     </row>
@@ -38287,16 +38311,16 @@
       <c r="C11" t="str">
         <v>Inavolu-Amaravathi</v>
       </c>
-      <c r="D11" t="str">
+      <c r="E11" t="str">
         <v>Subrmaniyam</v>
       </c>
-      <c r="E11" t="str">
+      <c r="F11" t="str">
         <v>IT Manager</v>
       </c>
-      <c r="F11" t="str">
+      <c r="G11" t="str">
         <v>9884492740</v>
       </c>
-      <c r="G11" t="str">
+      <c r="H11" t="str">
         <v>datacenter@srmap.edu.in</v>
       </c>
     </row>
@@ -38310,16 +38334,16 @@
       <c r="C12" t="str">
         <v>AP Secretariat</v>
       </c>
-      <c r="D12" t="str">
+      <c r="E12" t="str">
         <v>Sivaram</v>
       </c>
-      <c r="E12" t="str">
+      <c r="F12" t="str">
         <v>IT Manager</v>
       </c>
-      <c r="F12" t="str">
+      <c r="G12" t="str">
         <v>9550987700</v>
       </c>
-      <c r="G12" t="str">
+      <c r="H12" t="str">
         <v>tm-apscan@ap.gov.in</v>
       </c>
     </row>
@@ -38333,13 +38357,13 @@
       <c r="C13" t="str">
         <v>AP Secretariat</v>
       </c>
-      <c r="D13" t="str">
+      <c r="E13" t="str">
         <v>Naqueeb</v>
       </c>
-      <c r="E13" t="str">
+      <c r="F13" t="str">
         <v>IT staff</v>
       </c>
-      <c r="F13" t="str">
+      <c r="G13" t="str">
         <v>8328301237</v>
       </c>
     </row>
@@ -38353,13 +38377,13 @@
       <c r="C14" t="str">
         <v>AP Secretariat</v>
       </c>
-      <c r="D14" t="str">
+      <c r="E14" t="str">
         <v>Rajesh</v>
       </c>
-      <c r="E14" t="str">
+      <c r="F14" t="str">
         <v>IT staff</v>
       </c>
-      <c r="F14" t="str">
+      <c r="G14" t="str">
         <v>9908696681</v>
       </c>
     </row>
@@ -38373,16 +38397,16 @@
       <c r="C15" t="str">
         <v>AP Secretariat</v>
       </c>
-      <c r="D15" t="str">
+      <c r="E15" t="str">
         <v>Sreenivas Chirla</v>
       </c>
-      <c r="E15" t="str">
+      <c r="F15" t="str">
         <v>IT Director PA</v>
       </c>
-      <c r="F15" t="str">
+      <c r="G15" t="str">
         <v>8008040480</v>
       </c>
-      <c r="G15" t="str">
+      <c r="H15" t="str">
         <v>consultant-infra-itc@ap.gov.in</v>
       </c>
     </row>
@@ -38396,13 +38420,13 @@
       <c r="C16" t="str">
         <v>AP Secretariat</v>
       </c>
-      <c r="D16" t="str">
+      <c r="E16" t="str">
         <v>Manikanta</v>
       </c>
-      <c r="E16" t="str">
+      <c r="F16" t="str">
         <v>IT staff</v>
       </c>
-      <c r="F16" t="str">
+      <c r="G16" t="str">
         <v>9493151563</v>
       </c>
     </row>
@@ -38416,16 +38440,16 @@
       <c r="C17" t="str">
         <v>APTS-Vijayawada</v>
       </c>
-      <c r="D17" t="str">
+      <c r="E17" t="str">
         <v>Sridhar Reddy</v>
       </c>
-      <c r="E17" t="str">
+      <c r="F17" t="str">
         <v>Technical Consultant</v>
       </c>
-      <c r="F17" t="str">
+      <c r="G17" t="str">
         <v>9963029412</v>
       </c>
-      <c r="G17" t="str">
+      <c r="H17" t="str">
         <v>Sreedharreddy.A@gov.in</v>
       </c>
     </row>
@@ -38439,16 +38463,16 @@
       <c r="C18" t="str">
         <v>APTS-Vijayawada</v>
       </c>
-      <c r="D18" t="str">
+      <c r="E18" t="str">
         <v>Sailaja M</v>
       </c>
-      <c r="E18" t="str">
+      <c r="F18" t="str">
         <v>IT Manager</v>
       </c>
-      <c r="F18" t="str">
+      <c r="G18" t="str">
         <v>8474756522</v>
       </c>
-      <c r="G18" t="str">
+      <c r="H18" t="str">
         <v>msailaja-ap@nic.in</v>
       </c>
     </row>
@@ -38462,16 +38486,16 @@
       <c r="C19" t="str">
         <v>APTS-Vijayawada</v>
       </c>
-      <c r="D19" t="str">
+      <c r="E19" t="str">
         <v>Chalapathi Dasari</v>
       </c>
-      <c r="E19" t="str">
+      <c r="F19" t="str">
         <v>Clerk</v>
       </c>
-      <c r="F19" t="str">
+      <c r="G19" t="str">
         <v>9030110410</v>
       </c>
-      <c r="G19" t="str">
+      <c r="H19" t="str">
         <v>deo-iip-apts@ap.gov.in</v>
       </c>
     </row>
@@ -38485,10 +38509,10 @@
       <c r="C20" t="str">
         <v>APTS-Vijayawada</v>
       </c>
-      <c r="E20" t="str">
+      <c r="F20" t="str">
         <v>MD APTS</v>
       </c>
-      <c r="G20" t="str">
+      <c r="H20" t="str">
         <v>md_apts@ap.gov.in</v>
       </c>
     </row>
@@ -38502,13 +38526,13 @@
       <c r="C21" t="str">
         <v>AP Secretariat</v>
       </c>
-      <c r="D21" t="str">
+      <c r="E21" t="str">
         <v>D Venkatachalam</v>
       </c>
-      <c r="E21" t="str">
+      <c r="F21" t="str">
         <v>Director ITE&amp;C</v>
       </c>
-      <c r="G21" t="str">
+      <c r="H21" t="str">
         <v>dv.chalam@ap.gov.in</v>
       </c>
     </row>
@@ -38522,16 +38546,16 @@
       <c r="C22" t="str">
         <v>AP Secretariat</v>
       </c>
-      <c r="D22" t="str">
+      <c r="E22" t="str">
         <v>K Dhavuryan Naik</v>
       </c>
-      <c r="E22" t="str">
+      <c r="F22" t="str">
         <v>Director ITE&amp;C</v>
       </c>
-      <c r="F22" t="str">
+      <c r="G22" t="str">
         <v>9963029418</v>
       </c>
-      <c r="G22" t="str">
+      <c r="H22" t="str">
         <v>dir_comm_itc@ap.gov.in</v>
       </c>
     </row>
@@ -38545,16 +38569,16 @@
       <c r="C23" t="str">
         <v>APTS-Vijayawada</v>
       </c>
-      <c r="D23" t="str">
+      <c r="E23" t="str">
         <v>G.Vinod Kumar</v>
       </c>
-      <c r="E23" t="str">
+      <c r="F23" t="str">
         <v>Clerk</v>
       </c>
-      <c r="F23" t="str">
+      <c r="G23" t="str">
         <v>9491113416</v>
       </c>
-      <c r="G23" t="str">
+      <c r="H23" t="str">
         <v>vinodkumar.g16@nic.in</v>
       </c>
     </row>
@@ -38568,10 +38592,10 @@
       <c r="C24" t="str">
         <v>Rayapudi</v>
       </c>
-      <c r="D24" t="str">
+      <c r="E24" t="str">
         <v>Ajay</v>
       </c>
-      <c r="F24" t="str">
+      <c r="G24" t="str">
         <v>9886799510</v>
       </c>
     </row>
@@ -38585,13 +38609,13 @@
       <c r="C25" t="str">
         <v>Rayapudi</v>
       </c>
-      <c r="D25" t="str">
+      <c r="E25" t="str">
         <v>Ramesh</v>
       </c>
-      <c r="F25" t="str">
+      <c r="G25" t="str">
         <v>7095599100</v>
       </c>
-      <c r="G25" t="str">
+      <c r="H25" t="str">
         <v>ramesh@apcrda.org</v>
       </c>
     </row>
@@ -38605,13 +38629,13 @@
       <c r="C26" t="str">
         <v>Rayapudi</v>
       </c>
-      <c r="D26" t="str">
+      <c r="E26" t="str">
         <v>Teja</v>
       </c>
-      <c r="F26" t="str">
+      <c r="G26" t="str">
         <v>7095599078</v>
       </c>
-      <c r="G26" t="str">
+      <c r="H26" t="str">
         <v>itsupport@apcrda.org</v>
       </c>
     </row>
@@ -38625,13 +38649,13 @@
       <c r="C27" t="str">
         <v>Rayapudi</v>
       </c>
-      <c r="D27" t="str">
+      <c r="E27" t="str">
         <v>Yarshad</v>
       </c>
-      <c r="F27" t="str">
+      <c r="G27" t="str">
         <v>8008344994</v>
       </c>
-      <c r="G27" t="str">
+      <c r="H27" t="str">
         <v>itsupport@apcrda.org</v>
       </c>
     </row>
@@ -38645,13 +38669,13 @@
       <c r="C28" t="str">
         <v>Rayapudi</v>
       </c>
-      <c r="D28" t="str">
+      <c r="E28" t="str">
         <v>saritha</v>
       </c>
-      <c r="F28" t="str">
+      <c r="G28" t="str">
         <v>7095599848</v>
       </c>
-      <c r="G28" t="str">
+      <c r="H28" t="str">
         <v>itsupport@apcrda.org</v>
       </c>
     </row>
@@ -38665,16 +38689,16 @@
       <c r="C29" t="str">
         <v>Rayapudi</v>
       </c>
-      <c r="D29" t="str">
+      <c r="E29" t="str">
         <v>Lakshmi Prasanna</v>
       </c>
-      <c r="E29" t="str">
+      <c r="F29" t="str">
         <v>PM IT</v>
       </c>
-      <c r="F29" t="str">
+      <c r="G29" t="str">
         <v>7995015782</v>
       </c>
-      <c r="G29" t="str">
+      <c r="H29" t="str">
         <v>prasanna.m@apcrda.org</v>
       </c>
     </row>
@@ -38688,13 +38712,13 @@
       <c r="C30" t="str">
         <v>Rayapudi</v>
       </c>
-      <c r="D30" t="str">
+      <c r="E30" t="str">
         <v>Nadumpalli Srinivas</v>
       </c>
-      <c r="E30" t="str">
+      <c r="F30" t="str">
         <v>PA to Comissioner</v>
       </c>
-      <c r="F30" t="str">
+      <c r="G30" t="str">
         <v>7095599822</v>
       </c>
     </row>
@@ -38708,16 +38732,16 @@
       <c r="C31" t="str">
         <v>Nelapadu Amaravathi</v>
       </c>
-      <c r="D31" t="str">
+      <c r="E31" t="str">
         <v>Edukondalu</v>
       </c>
-      <c r="E31" t="str">
+      <c r="F31" t="str">
         <v>Registrar IT</v>
       </c>
-      <c r="F31" t="str">
+      <c r="G31" t="str">
         <v>7901625203 9848455669</v>
       </c>
-      <c r="G31" t="str">
+      <c r="H31" t="str">
         <v>cpc-ap@aij.gov.in</v>
       </c>
     </row>
@@ -38731,13 +38755,13 @@
       <c r="C32" t="str">
         <v>Nelapadu Amaravathi</v>
       </c>
-      <c r="D32" t="str">
+      <c r="E32" t="str">
         <v>Hussain vali</v>
       </c>
-      <c r="E32" t="str">
+      <c r="F32" t="str">
         <v>Registrar IT staff</v>
       </c>
-      <c r="F32" t="str">
+      <c r="G32" t="str">
         <v>9515000616</v>
       </c>
     </row>
@@ -38751,10 +38775,10 @@
       <c r="C33" t="str">
         <v>Nelapadu Amaravathi</v>
       </c>
-      <c r="D33" t="str">
+      <c r="E33" t="str">
         <v>Mobeen</v>
       </c>
-      <c r="E33" t="str">
+      <c r="F33" t="str">
         <v>Registrar IT staff</v>
       </c>
     </row>
@@ -38768,13 +38792,13 @@
       <c r="C34" t="str">
         <v>Nelapadu Amaravathi</v>
       </c>
-      <c r="D34" t="str">
+      <c r="E34" t="str">
         <v>Venkata Ramana</v>
       </c>
-      <c r="E34" t="str">
+      <c r="F34" t="str">
         <v>ASST registarar</v>
       </c>
-      <c r="F34" t="str">
+      <c r="G34" t="str">
         <v>9494777799 7901625189 7569458775</v>
       </c>
     </row>
@@ -38788,13 +38812,13 @@
       <c r="C35" t="str">
         <v>Nelapadu Amaravathi</v>
       </c>
-      <c r="D35" t="str">
+      <c r="E35" t="str">
         <v>Suresh</v>
       </c>
-      <c r="E35" t="str">
+      <c r="F35" t="str">
         <v>JL section -LL related</v>
       </c>
-      <c r="F35" t="str">
+      <c r="G35" t="str">
         <v>9985557738</v>
       </c>
     </row>
@@ -38808,22 +38832,22 @@
       <c r="C36" t="str">
         <v>opposit Secretariat</v>
       </c>
-      <c r="D36" t="str">
+      <c r="E36" t="str">
         <v>N J Rao</v>
       </c>
-      <c r="E36" t="str">
+      <c r="F36" t="str">
         <v>Adminstrative officer</v>
       </c>
-      <c r="F36" t="str">
+      <c r="G36" t="str">
         <v>9440621433 9849682103</v>
       </c>
-      <c r="G36" t="str">
+      <c r="H36" t="str">
         <v>apslsauthority@yahoo.com</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O36"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>